<commit_message>
refactor: ajustar estrutura da planilha
</commit_message>
<xml_diff>
--- a/src/truckdwell/assets/planilha_estadia.xlsx
+++ b/src/truckdwell/assets/planilha_estadia.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="25">
   <si>
     <t xml:space="preserve">Cálculo de Estadia</t>
   </si>
@@ -99,21 +99,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SALITRE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CARVALHO TRANSPORTES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROCHA CMISS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JOSÉ CARLOS XAVIER DA SILVA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTIVO: ACÚMULO DE VEÍCULOS</t>
   </si>
 </sst>
 </file>
@@ -372,104 +357,108 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -477,75 +466,75 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -804,254 +793,254 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="3.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="3.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="5"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="9"/>
+      <c r="E3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="5"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="12" t="n">
         <v>2486</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>44539</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="10" t="s">
+      <c r="D5" s="9"/>
+      <c r="E5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-      <c r="B6" s="14" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <f aca="true">TODAY()</f>
-        <v>45953</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="10" t="s">
+        <v>45971</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="5"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="14" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="5"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4"/>
-      <c r="B9" s="21" t="n">
+      <c r="A9" s="5"/>
+      <c r="B9" s="22" t="n">
         <v>45434.6576388889</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="5"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="6" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="G10" s="23"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-      <c r="B11" s="24" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="10" t="s">
+      <c r="C11" s="25"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">(B15-B12)*24</f>
         <v>36.2500000001164</v>
       </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="5"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="26" t="n">
+      <c r="A12" s="5"/>
+      <c r="B12" s="27" t="n">
         <f aca="false">B9+0.5</f>
         <v>45435.1576388889</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="10" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <v>45.39</v>
       </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="5"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="14" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="29" t="n">
         <f aca="false">F10*F11*F12</f>
         <v>822.693750002642</v>
       </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="5"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="20" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="29" t="s">
+      <c r="C14" s="21"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="5"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="30" t="n">
+      <c r="A15" s="5"/>
+      <c r="B15" s="31" t="n">
         <v>45436.6680555556</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8" t="s">
+      <c r="C15" s="31"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="8"/>
-      <c r="H15" s="5"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="31"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="32"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="34"/>
+      <c r="A17" s="33"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1086,254 +1075,254 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="3.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="3.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="5"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="9"/>
+      <c r="E3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="5"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="12" t="n">
         <v>2486</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>44539</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="10" t="s">
+      <c r="D5" s="9"/>
+      <c r="E5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-      <c r="B6" s="14" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <f aca="true">TODAY()</f>
-        <v>45953</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="10" t="s">
+        <v>45971</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="5"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="14" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="5"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4"/>
-      <c r="B9" s="21" t="n">
+      <c r="A9" s="5"/>
+      <c r="B9" s="22" t="n">
         <v>45434.6576388889</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="5"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="6" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="G10" s="23"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-      <c r="B11" s="24" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="10" t="s">
+      <c r="C11" s="25"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">(B15-B12)*24</f>
         <v>36.2500000001164</v>
       </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="5"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="26" t="n">
+      <c r="A12" s="5"/>
+      <c r="B12" s="27" t="n">
         <f aca="false">B9+0.5</f>
         <v>45435.1576388889</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="10" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <v>45.39</v>
       </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="5"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="14" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="29" t="n">
         <f aca="false">F10*F11*F12</f>
         <v>822.693750002642</v>
       </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="5"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="20" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="29" t="s">
+      <c r="C14" s="21"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="5"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="30" t="n">
+      <c r="A15" s="5"/>
+      <c r="B15" s="31" t="n">
         <v>45436.6680555556</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8" t="s">
+      <c r="C15" s="31"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="8"/>
-      <c r="H15" s="5"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="31"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="32"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="34"/>
+      <c r="A17" s="33"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1368,254 +1357,254 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="3.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="3.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="5"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="9"/>
+      <c r="E3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="5"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="12" t="n">
         <v>2486</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>44539</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="10" t="s">
+      <c r="D5" s="9"/>
+      <c r="E5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-      <c r="B6" s="14" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <f aca="true">TODAY()</f>
-        <v>45953</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="10" t="s">
+        <v>45971</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="5"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="14" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="5"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4"/>
-      <c r="B9" s="21" t="n">
+      <c r="A9" s="5"/>
+      <c r="B9" s="22" t="n">
         <v>45434.6576388889</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="5"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="6" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="G10" s="23"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-      <c r="B11" s="24" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="10" t="s">
+      <c r="C11" s="25"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">(B15-B12)*24</f>
         <v>36.2500000001164</v>
       </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="5"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="26" t="n">
+      <c r="A12" s="5"/>
+      <c r="B12" s="27" t="n">
         <f aca="false">B9+0.5</f>
         <v>45435.1576388889</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="10" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <v>45.39</v>
       </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="5"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="14" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="29" t="n">
         <f aca="false">F10*F11*F12</f>
         <v>822.693750002642</v>
       </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="5"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="20" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="29" t="s">
+      <c r="C14" s="21"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="5"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="30" t="n">
+      <c r="A15" s="5"/>
+      <c r="B15" s="31" t="n">
         <v>45436.6680555556</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8" t="s">
+      <c r="C15" s="31"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="8"/>
-      <c r="H15" s="5"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="31"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="32"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="34"/>
+      <c r="A17" s="33"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1650,254 +1639,254 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="3.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="3.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="5"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="9"/>
+      <c r="E3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="5"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="12" t="n">
         <v>2486</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>44539</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="10" t="s">
+      <c r="D5" s="9"/>
+      <c r="E5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-      <c r="B6" s="14" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <f aca="true">TODAY()</f>
-        <v>45953</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="10" t="s">
+        <v>45971</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="5"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="14" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="5"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4"/>
-      <c r="B9" s="21" t="n">
+      <c r="A9" s="5"/>
+      <c r="B9" s="22" t="n">
         <v>45434.6576388889</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="5"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="6" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="G10" s="23"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-      <c r="B11" s="24" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="10" t="s">
+      <c r="C11" s="25"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">(B15-B12)*24</f>
         <v>36.2500000001164</v>
       </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="5"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="26" t="n">
+      <c r="A12" s="5"/>
+      <c r="B12" s="27" t="n">
         <f aca="false">B9+0.5</f>
         <v>45435.1576388889</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="10" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <v>45.39</v>
       </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="5"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="14" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="29" t="n">
         <f aca="false">F10*F11*F12</f>
         <v>822.693750002642</v>
       </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="5"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="20" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="29" t="s">
+      <c r="C14" s="21"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="5"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="30" t="n">
+      <c r="A15" s="5"/>
+      <c r="B15" s="31" t="n">
         <v>45436.6680555556</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8" t="s">
+      <c r="C15" s="31"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="8"/>
-      <c r="H15" s="5"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="31"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="32"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="34"/>
+      <c r="A17" s="33"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1932,264 +1921,245 @@
   <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="3.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="3.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="5"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="6" t="s">
+      <c r="C3" s="36"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="5"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="37" t="n">
-        <v>20020</v>
-      </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="10" t="s">
+      <c r="C4" s="38"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="38" t="n">
-        <v>152</v>
-      </c>
-      <c r="G4" s="39"/>
-      <c r="H4" s="5"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="10" t="s">
+      <c r="C5" s="40"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="39"/>
-      <c r="H5" s="5"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-      <c r="B6" s="14" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="40" t="n">
+      <c r="C6" s="41" t="n">
         <f aca="true">TODAY()</f>
-        <v>45953</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="10" t="s">
+        <v>45971</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="5"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="14" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="5"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4"/>
-      <c r="B9" s="41" t="n">
-        <v>45519.8777777778</v>
-      </c>
-      <c r="C9" s="41"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="5"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="6" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="G10" s="23"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4"/>
-      <c r="B11" s="24" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="10" t="s">
+      <c r="C11" s="25"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">(B15-B12)*24</f>
-        <v>41.233333333279</v>
-      </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="5"/>
+        <v>-12</v>
+      </c>
+      <c r="G11" s="26"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4"/>
-      <c r="B12" s="26" t="n">
+      <c r="A12" s="5"/>
+      <c r="B12" s="27" t="n">
         <f aca="false">B9+0.5</f>
-        <v>45520.3777777778</v>
-      </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="10" t="s">
+        <v>0.5</v>
+      </c>
+      <c r="C12" s="27"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="42" t="n">
-        <v>47.08</v>
-      </c>
-      <c r="G12" s="42"/>
-      <c r="H12" s="5"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="14" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="28" t="n">
+      <c r="F13" s="29" t="n">
         <f aca="false">F10*F11*F12</f>
-        <v>970.632666665388</v>
-      </c>
-      <c r="G13" s="28"/>
-      <c r="H13" s="5"/>
+        <v>-0</v>
+      </c>
+      <c r="G13" s="29"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="20" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="8"/>
-      <c r="H14" s="5"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="9"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
-      <c r="B15" s="41" t="n">
-        <v>45522.0958333333</v>
-      </c>
-      <c r="C15" s="41"/>
-      <c r="D15" s="8"/>
-      <c r="H15" s="5"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="9"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="43" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="5"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="44"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4"/>
-      <c r="E17" s="8" t="s">
+      <c r="A17" s="5"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="9"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="E18" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="G17" s="8"/>
-      <c r="H17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4"/>
-      <c r="H18" s="5"/>
+      <c r="H18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
-      <c r="H19" s="5"/>
+      <c r="A19" s="5"/>
+      <c r="H19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="32"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="34"/>
+      <c r="A20" s="33"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>